<commit_message>
Update Trafic.xlsx with the latest traffic data.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Trafic.xlsx
+++ b/Trafic.xlsx
@@ -9,17 +9,21 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="4294939905" windowHeight="16725" tabRatio="500"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="4294939905" windowHeight="16725" tabRatio="500" activeTab="1"/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <x:sheet name="등교 시간" sheetId="1" r:id="rId4"/>
+    <x:sheet name="하교 시간" sheetId="2" r:id="rId5"/>
   </x:sheets>
   <x:calcPr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" mc:Ignorable="hs" hs:hclCalcId="904"/>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="8">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="10">
+  <x:si>
+    <x:t>초</x:t>
+  </x:si>
   <x:si>
     <x:t>시</x:t>
   </x:si>
@@ -30,19 +34,22 @@
     <x:t>롯데마트 사거리</x:t>
   </x:si>
   <x:si>
+    <x:t>보평초교 사거리</x:t>
+  </x:si>
+  <x:si>
     <x:t>보평초 정문앞 신호등</x:t>
   </x:si>
   <x:si>
-    <x:t>보평초교 사거리</x:t>
+    <x:t>빨간불 시작</x:t>
   </x:si>
   <x:si>
     <x:t>초록불 시작</x:t>
   </x:si>
   <x:si>
-    <x:t>빨간불 시작</x:t>
+    <x:t>구숯내 삼거리</x:t>
   </x:si>
   <x:si>
-    <x:t>초</x:t>
+    <x:t>1단지 앞 신호등</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -110,7 +117,7 @@
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
@@ -140,6 +147,9 @@
         </x:xf>
       </mc:Fallback>
     </mc:AlternateContent>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
         <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" hs:applyExtension="1">
@@ -475,64 +485,69 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:J34"/>
+  <x:dimension ref="A1:M34"/>
   <x:sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.39999999999999857891"/>
   <x:cols>
     <x:col min="1" max="1" width="11.75390625" customWidth="1"/>
     <x:col min="2" max="10" width="12.25390625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:10">
+    <x:row r="1" spans="1:13">
       <x:c r="A1" s="1"/>
-      <x:c r="B1" s="3" t="s">
+      <x:c r="B1" s="4" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3" t="s">
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
     </x:row>
     <x:row r="2" spans="1:10">
       <x:c r="A2" s="1"/>
       <x:c r="B2" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="E2" s="2" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="E2" s="2" t="s">
+      <x:c r="F2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="s">
+      <x:c r="H2" s="2" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H2" s="2" t="s">
+      <x:c r="I2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J2" s="1" t="s">
         <x:v>0</x:v>
-      </x:c>
-      <x:c r="I2" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J2" s="1" t="s">
-        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:10">
       <x:c r="A3" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -560,7 +575,7 @@
     </x:row>
     <x:row r="5" spans="1:10">
       <x:c r="A5" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B5" s="1"/>
       <x:c r="C5" s="1"/>
@@ -588,7 +603,7 @@
     </x:row>
     <x:row r="7" spans="1:10">
       <x:c r="A7" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -616,7 +631,7 @@
     </x:row>
     <x:row r="9" spans="1:10">
       <x:c r="A9" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="1"/>
@@ -644,7 +659,7 @@
     </x:row>
     <x:row r="11" spans="1:10">
       <x:c r="A11" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B11" s="1"/>
       <x:c r="C11" s="1"/>
@@ -672,7 +687,7 @@
     </x:row>
     <x:row r="13" spans="1:10">
       <x:c r="A13" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B13" s="1"/>
       <x:c r="C13" s="1"/>
@@ -700,7 +715,7 @@
     </x:row>
     <x:row r="15" spans="1:10">
       <x:c r="A15" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B15" s="1"/>
       <x:c r="C15" s="1"/>
@@ -728,7 +743,7 @@
     </x:row>
     <x:row r="17" spans="1:10">
       <x:c r="A17" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B17" s="1"/>
       <x:c r="C17" s="1"/>
@@ -756,7 +771,7 @@
     </x:row>
     <x:row r="19" spans="1:10">
       <x:c r="A19" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B19" s="1"/>
       <x:c r="C19" s="1"/>
@@ -784,7 +799,7 @@
     </x:row>
     <x:row r="21" spans="1:10">
       <x:c r="A21" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B21" s="1"/>
       <x:c r="C21" s="1"/>
@@ -812,7 +827,7 @@
     </x:row>
     <x:row r="23" spans="1:10">
       <x:c r="A23" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B23" s="1"/>
       <x:c r="C23" s="1"/>
@@ -840,7 +855,7 @@
     </x:row>
     <x:row r="25" spans="1:10">
       <x:c r="A25" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B25" s="1"/>
       <x:c r="C25" s="1"/>
@@ -868,7 +883,7 @@
     </x:row>
     <x:row r="27" spans="1:10">
       <x:c r="A27" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B27" s="1"/>
       <x:c r="C27" s="1"/>
@@ -896,7 +911,7 @@
     </x:row>
     <x:row r="29" spans="1:10">
       <x:c r="A29" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B29" s="1"/>
       <x:c r="C29" s="1"/>
@@ -924,7 +939,7 @@
     </x:row>
     <x:row r="31" spans="1:10">
       <x:c r="A31" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B31" s="1"/>
       <x:c r="C31" s="1"/>
@@ -952,7 +967,7 @@
     </x:row>
     <x:row r="33" spans="1:10">
       <x:c r="A33" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B33" s="1"/>
       <x:c r="C33" s="1"/>
@@ -979,13 +994,685 @@
       <x:c r="J34" s="1"/>
     </x:row>
   </x:sheetData>
-  <x:mergeCells count="3">
+  <x:mergeCells count="4">
     <x:mergeCell ref="B1:D1"/>
     <x:mergeCell ref="E1:G1"/>
     <x:mergeCell ref="H1:J1"/>
+    <x:mergeCell ref="K1:M1"/>
   </x:mergeCells>
-  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51180553436279296875" footer="0.51180553436279296875"/>
+  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51138889789581298828" footer="0.51138889789581298828"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="0" fitToHeight="0" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="0" verticalDpi="0" copies="1"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr codeName="Sheet2"/>
+  <x:dimension ref="A1:P40"/>
+  <x:sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.39999999999999857891"/>
+  <x:sheetData>
+    <x:row r="1" spans="1:16">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="4" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
+      <x:c r="N1" s="4" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="O1" s="4"/>
+      <x:c r="P1" s="4"/>
+    </x:row>
+    <x:row r="2" spans="1:16">
+      <x:c r="A2" s="1"/>
+      <x:c r="B2" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:13">
+      <x:c r="A3" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+      <x:c r="K3" s="3"/>
+      <x:c r="L3" s="3"/>
+      <x:c r="M3" s="3"/>
+    </x:row>
+    <x:row r="4" spans="1:13">
+      <x:c r="A4" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+      <x:c r="K4" s="3"/>
+      <x:c r="L4" s="3"/>
+      <x:c r="M4" s="3"/>
+    </x:row>
+    <x:row r="5" spans="1:13">
+      <x:c r="A5" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+      <x:c r="I5" s="1"/>
+      <x:c r="J5" s="1"/>
+      <x:c r="K5" s="3"/>
+      <x:c r="L5" s="3"/>
+      <x:c r="M5" s="3"/>
+    </x:row>
+    <x:row r="6" spans="1:13">
+      <x:c r="A6" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B6" s="1"/>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="1"/>
+      <x:c r="G6" s="1"/>
+      <x:c r="H6" s="1"/>
+      <x:c r="I6" s="1"/>
+      <x:c r="J6" s="1"/>
+      <x:c r="K6" s="3"/>
+      <x:c r="L6" s="3"/>
+      <x:c r="M6" s="3"/>
+    </x:row>
+    <x:row r="7" spans="1:13">
+      <x:c r="A7" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="1"/>
+      <x:c r="D7" s="1"/>
+      <x:c r="E7" s="1"/>
+      <x:c r="F7" s="1"/>
+      <x:c r="G7" s="1"/>
+      <x:c r="H7" s="1"/>
+      <x:c r="I7" s="1"/>
+      <x:c r="J7" s="1"/>
+      <x:c r="K7" s="3"/>
+      <x:c r="L7" s="3"/>
+      <x:c r="M7" s="3"/>
+    </x:row>
+    <x:row r="8" spans="1:13">
+      <x:c r="A8" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1"/>
+      <x:c r="D8" s="1"/>
+      <x:c r="E8" s="1"/>
+      <x:c r="F8" s="1"/>
+      <x:c r="G8" s="1"/>
+      <x:c r="H8" s="1"/>
+      <x:c r="I8" s="1"/>
+      <x:c r="J8" s="1"/>
+      <x:c r="K8" s="3"/>
+      <x:c r="L8" s="3"/>
+      <x:c r="M8" s="3"/>
+    </x:row>
+    <x:row r="9" spans="1:13">
+      <x:c r="A9" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1"/>
+      <x:c r="D9" s="1"/>
+      <x:c r="E9" s="1"/>
+      <x:c r="F9" s="1"/>
+      <x:c r="G9" s="1"/>
+      <x:c r="H9" s="1"/>
+      <x:c r="I9" s="1"/>
+      <x:c r="J9" s="1"/>
+      <x:c r="K9" s="3"/>
+      <x:c r="L9" s="3"/>
+      <x:c r="M9" s="3"/>
+    </x:row>
+    <x:row r="10" spans="1:13">
+      <x:c r="A10" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="1"/>
+      <x:c r="C10" s="1"/>
+      <x:c r="D10" s="1"/>
+      <x:c r="E10" s="1"/>
+      <x:c r="F10" s="1"/>
+      <x:c r="G10" s="1"/>
+      <x:c r="H10" s="1"/>
+      <x:c r="I10" s="1"/>
+      <x:c r="J10" s="1"/>
+      <x:c r="K10" s="3"/>
+      <x:c r="L10" s="3"/>
+      <x:c r="M10" s="3"/>
+    </x:row>
+    <x:row r="11" spans="1:13">
+      <x:c r="A11" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1"/>
+      <x:c r="D11" s="1"/>
+      <x:c r="E11" s="1"/>
+      <x:c r="F11" s="1"/>
+      <x:c r="G11" s="1"/>
+      <x:c r="H11" s="1"/>
+      <x:c r="I11" s="1"/>
+      <x:c r="J11" s="1"/>
+      <x:c r="K11" s="3"/>
+      <x:c r="L11" s="3"/>
+      <x:c r="M11" s="3"/>
+    </x:row>
+    <x:row r="12" spans="1:13">
+      <x:c r="A12" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="1"/>
+      <x:c r="E12" s="1"/>
+      <x:c r="F12" s="1"/>
+      <x:c r="G12" s="1"/>
+      <x:c r="H12" s="1"/>
+      <x:c r="I12" s="1"/>
+      <x:c r="J12" s="1"/>
+      <x:c r="K12" s="3"/>
+      <x:c r="L12" s="3"/>
+      <x:c r="M12" s="3"/>
+    </x:row>
+    <x:row r="13" spans="1:13">
+      <x:c r="A13" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B13" s="1"/>
+      <x:c r="C13" s="1"/>
+      <x:c r="D13" s="1"/>
+      <x:c r="E13" s="1"/>
+      <x:c r="F13" s="1"/>
+      <x:c r="G13" s="1"/>
+      <x:c r="H13" s="1"/>
+      <x:c r="I13" s="1"/>
+      <x:c r="J13" s="1"/>
+      <x:c r="K13" s="3"/>
+      <x:c r="L13" s="3"/>
+      <x:c r="M13" s="3"/>
+    </x:row>
+    <x:row r="14" spans="1:13">
+      <x:c r="A14" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="1"/>
+      <x:c r="E14" s="1"/>
+      <x:c r="F14" s="1"/>
+      <x:c r="G14" s="1"/>
+      <x:c r="H14" s="1"/>
+      <x:c r="I14" s="1"/>
+      <x:c r="J14" s="1"/>
+      <x:c r="K14" s="3"/>
+      <x:c r="L14" s="3"/>
+      <x:c r="M14" s="3"/>
+    </x:row>
+    <x:row r="15" spans="1:13">
+      <x:c r="A15" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B15" s="1"/>
+      <x:c r="C15" s="1"/>
+      <x:c r="D15" s="1"/>
+      <x:c r="E15" s="1"/>
+      <x:c r="F15" s="1"/>
+      <x:c r="G15" s="1"/>
+      <x:c r="H15" s="1"/>
+      <x:c r="I15" s="1"/>
+      <x:c r="J15" s="1"/>
+      <x:c r="K15" s="3"/>
+      <x:c r="L15" s="3"/>
+      <x:c r="M15" s="3"/>
+    </x:row>
+    <x:row r="16" spans="1:13">
+      <x:c r="A16" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B16" s="1"/>
+      <x:c r="C16" s="1"/>
+      <x:c r="D16" s="1"/>
+      <x:c r="E16" s="1"/>
+      <x:c r="F16" s="1"/>
+      <x:c r="G16" s="1"/>
+      <x:c r="H16" s="1"/>
+      <x:c r="I16" s="1"/>
+      <x:c r="J16" s="1"/>
+      <x:c r="K16" s="3"/>
+      <x:c r="L16" s="3"/>
+      <x:c r="M16" s="3"/>
+    </x:row>
+    <x:row r="17" spans="1:13">
+      <x:c r="A17" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1"/>
+      <x:c r="D17" s="1"/>
+      <x:c r="E17" s="1"/>
+      <x:c r="F17" s="1"/>
+      <x:c r="G17" s="1"/>
+      <x:c r="H17" s="1"/>
+      <x:c r="I17" s="1"/>
+      <x:c r="J17" s="1"/>
+      <x:c r="K17" s="3"/>
+      <x:c r="L17" s="3"/>
+      <x:c r="M17" s="3"/>
+    </x:row>
+    <x:row r="18" spans="1:13">
+      <x:c r="A18" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18" s="1"/>
+      <x:c r="D18" s="1"/>
+      <x:c r="E18" s="1"/>
+      <x:c r="F18" s="1"/>
+      <x:c r="G18" s="1"/>
+      <x:c r="H18" s="1"/>
+      <x:c r="I18" s="1"/>
+      <x:c r="J18" s="1"/>
+      <x:c r="K18" s="3"/>
+      <x:c r="L18" s="3"/>
+      <x:c r="M18" s="3"/>
+    </x:row>
+    <x:row r="19" spans="1:13">
+      <x:c r="A19" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B19" s="1"/>
+      <x:c r="C19" s="1"/>
+      <x:c r="D19" s="1"/>
+      <x:c r="E19" s="1"/>
+      <x:c r="F19" s="1"/>
+      <x:c r="G19" s="1"/>
+      <x:c r="H19" s="1"/>
+      <x:c r="I19" s="1"/>
+      <x:c r="J19" s="1"/>
+      <x:c r="K19" s="3"/>
+      <x:c r="L19" s="3"/>
+      <x:c r="M19" s="3"/>
+    </x:row>
+    <x:row r="20" spans="1:13">
+      <x:c r="A20" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B20" s="1"/>
+      <x:c r="C20" s="1"/>
+      <x:c r="D20" s="1"/>
+      <x:c r="E20" s="1"/>
+      <x:c r="F20" s="1"/>
+      <x:c r="G20" s="1"/>
+      <x:c r="H20" s="1"/>
+      <x:c r="I20" s="1"/>
+      <x:c r="J20" s="1"/>
+      <x:c r="K20" s="3"/>
+      <x:c r="L20" s="3"/>
+      <x:c r="M20" s="3"/>
+    </x:row>
+    <x:row r="21" spans="1:13">
+      <x:c r="A21" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B21" s="1"/>
+      <x:c r="C21" s="1"/>
+      <x:c r="D21" s="1"/>
+      <x:c r="E21" s="1"/>
+      <x:c r="F21" s="1"/>
+      <x:c r="G21" s="1"/>
+      <x:c r="H21" s="1"/>
+      <x:c r="I21" s="1"/>
+      <x:c r="J21" s="1"/>
+      <x:c r="K21" s="3"/>
+      <x:c r="L21" s="3"/>
+      <x:c r="M21" s="3"/>
+    </x:row>
+    <x:row r="22" spans="1:13">
+      <x:c r="A22" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B22" s="1"/>
+      <x:c r="C22" s="1"/>
+      <x:c r="D22" s="1"/>
+      <x:c r="E22" s="1"/>
+      <x:c r="F22" s="1"/>
+      <x:c r="G22" s="1"/>
+      <x:c r="H22" s="1"/>
+      <x:c r="I22" s="1"/>
+      <x:c r="J22" s="1"/>
+      <x:c r="K22" s="3"/>
+      <x:c r="L22" s="3"/>
+      <x:c r="M22" s="3"/>
+    </x:row>
+    <x:row r="23" spans="1:13">
+      <x:c r="A23" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B23" s="1"/>
+      <x:c r="C23" s="1"/>
+      <x:c r="D23" s="1"/>
+      <x:c r="E23" s="1"/>
+      <x:c r="F23" s="1"/>
+      <x:c r="G23" s="1"/>
+      <x:c r="H23" s="1"/>
+      <x:c r="I23" s="1"/>
+      <x:c r="J23" s="1"/>
+      <x:c r="K23" s="3"/>
+      <x:c r="L23" s="3"/>
+      <x:c r="M23" s="3"/>
+    </x:row>
+    <x:row r="24" spans="1:13">
+      <x:c r="A24" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B24" s="1"/>
+      <x:c r="C24" s="1"/>
+      <x:c r="D24" s="1"/>
+      <x:c r="E24" s="1"/>
+      <x:c r="F24" s="1"/>
+      <x:c r="G24" s="1"/>
+      <x:c r="H24" s="1"/>
+      <x:c r="I24" s="1"/>
+      <x:c r="J24" s="1"/>
+      <x:c r="K24" s="3"/>
+      <x:c r="L24" s="3"/>
+      <x:c r="M24" s="3"/>
+    </x:row>
+    <x:row r="25" spans="1:13">
+      <x:c r="A25" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B25" s="1"/>
+      <x:c r="C25" s="1"/>
+      <x:c r="D25" s="1"/>
+      <x:c r="E25" s="1"/>
+      <x:c r="F25" s="1"/>
+      <x:c r="G25" s="1"/>
+      <x:c r="H25" s="1"/>
+      <x:c r="I25" s="1"/>
+      <x:c r="J25" s="1"/>
+      <x:c r="K25" s="3"/>
+      <x:c r="L25" s="3"/>
+      <x:c r="M25" s="3"/>
+    </x:row>
+    <x:row r="26" spans="1:13">
+      <x:c r="A26" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B26" s="1"/>
+      <x:c r="C26" s="1"/>
+      <x:c r="D26" s="1"/>
+      <x:c r="E26" s="1"/>
+      <x:c r="F26" s="1"/>
+      <x:c r="G26" s="1"/>
+      <x:c r="H26" s="1"/>
+      <x:c r="I26" s="1"/>
+      <x:c r="J26" s="1"/>
+      <x:c r="K26" s="3"/>
+      <x:c r="L26" s="3"/>
+      <x:c r="M26" s="3"/>
+    </x:row>
+    <x:row r="27" spans="1:13">
+      <x:c r="A27" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B27" s="1"/>
+      <x:c r="C27" s="1"/>
+      <x:c r="D27" s="1"/>
+      <x:c r="E27" s="1"/>
+      <x:c r="F27" s="1"/>
+      <x:c r="G27" s="1"/>
+      <x:c r="H27" s="1"/>
+      <x:c r="I27" s="1"/>
+      <x:c r="J27" s="1"/>
+      <x:c r="K27" s="3"/>
+      <x:c r="L27" s="3"/>
+      <x:c r="M27" s="3"/>
+    </x:row>
+    <x:row r="28" spans="1:13">
+      <x:c r="A28" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B28" s="1"/>
+      <x:c r="C28" s="1"/>
+      <x:c r="D28" s="1"/>
+      <x:c r="E28" s="1"/>
+      <x:c r="F28" s="1"/>
+      <x:c r="G28" s="1"/>
+      <x:c r="H28" s="1"/>
+      <x:c r="I28" s="1"/>
+      <x:c r="J28" s="1"/>
+      <x:c r="K28" s="3"/>
+      <x:c r="L28" s="3"/>
+      <x:c r="M28" s="3"/>
+    </x:row>
+    <x:row r="29" spans="1:13">
+      <x:c r="A29" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B29" s="1"/>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="1"/>
+      <x:c r="E29" s="1"/>
+      <x:c r="F29" s="1"/>
+      <x:c r="G29" s="1"/>
+      <x:c r="H29" s="1"/>
+      <x:c r="I29" s="1"/>
+      <x:c r="J29" s="1"/>
+      <x:c r="K29" s="3"/>
+      <x:c r="L29" s="3"/>
+      <x:c r="M29" s="3"/>
+    </x:row>
+    <x:row r="30" spans="1:13">
+      <x:c r="A30" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B30" s="1"/>
+      <x:c r="C30" s="1"/>
+      <x:c r="D30" s="1"/>
+      <x:c r="E30" s="1"/>
+      <x:c r="F30" s="1"/>
+      <x:c r="G30" s="1"/>
+      <x:c r="H30" s="1"/>
+      <x:c r="I30" s="1"/>
+      <x:c r="J30" s="1"/>
+      <x:c r="K30" s="3"/>
+      <x:c r="L30" s="3"/>
+      <x:c r="M30" s="3"/>
+    </x:row>
+    <x:row r="31" spans="1:13">
+      <x:c r="A31" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B31" s="1"/>
+      <x:c r="C31" s="1"/>
+      <x:c r="D31" s="1"/>
+      <x:c r="E31" s="1"/>
+      <x:c r="F31" s="1"/>
+      <x:c r="G31" s="1"/>
+      <x:c r="H31" s="1"/>
+      <x:c r="I31" s="1"/>
+      <x:c r="J31" s="1"/>
+      <x:c r="K31" s="3"/>
+      <x:c r="L31" s="3"/>
+      <x:c r="M31" s="3"/>
+    </x:row>
+    <x:row r="32" spans="1:13">
+      <x:c r="A32" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B32" s="1"/>
+      <x:c r="C32" s="1"/>
+      <x:c r="D32" s="1"/>
+      <x:c r="E32" s="1"/>
+      <x:c r="F32" s="1"/>
+      <x:c r="G32" s="1"/>
+      <x:c r="H32" s="1"/>
+      <x:c r="I32" s="1"/>
+      <x:c r="J32" s="1"/>
+      <x:c r="K32" s="3"/>
+      <x:c r="L32" s="3"/>
+      <x:c r="M32" s="3"/>
+    </x:row>
+    <x:row r="33" spans="1:13">
+      <x:c r="A33" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B33" s="1"/>
+      <x:c r="C33" s="1"/>
+      <x:c r="D33" s="1"/>
+      <x:c r="E33" s="1"/>
+      <x:c r="F33" s="1"/>
+      <x:c r="G33" s="1"/>
+      <x:c r="H33" s="1"/>
+      <x:c r="I33" s="1"/>
+      <x:c r="J33" s="1"/>
+      <x:c r="K33" s="3"/>
+      <x:c r="L33" s="3"/>
+      <x:c r="M33" s="3"/>
+    </x:row>
+    <x:row r="34" spans="1:13">
+      <x:c r="A34" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B34" s="1"/>
+      <x:c r="C34" s="1"/>
+      <x:c r="D34" s="1"/>
+      <x:c r="E34" s="1"/>
+      <x:c r="F34" s="1"/>
+      <x:c r="G34" s="1"/>
+      <x:c r="H34" s="1"/>
+      <x:c r="I34" s="1"/>
+      <x:c r="J34" s="1"/>
+      <x:c r="K34" s="3"/>
+      <x:c r="L34" s="3"/>
+      <x:c r="M34" s="3"/>
+    </x:row>
+    <x:row r="35" spans="1:1">
+      <x:c r="A35" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:1">
+      <x:c r="A36" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" spans="1:1">
+      <x:c r="A37" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:1">
+      <x:c r="A38" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:1">
+      <x:c r="A39" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" spans="1:1">
+      <x:c r="A40" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells count="5">
+    <x:mergeCell ref="B1:D1"/>
+    <x:mergeCell ref="E1:G1"/>
+    <x:mergeCell ref="H1:J1"/>
+    <x:mergeCell ref="K1:M1"/>
+    <x:mergeCell ref="N1:P1"/>
+  </x:mergeCells>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="1" gridLinesSet="1"/>
+  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51152777671813964844" footer="0.51152777671813964844"/>
+  <x:pageSetup paperSize="9" scale="74" firstPageNumber="1" fitToWidth="0" fitToHeight="0" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="0" verticalDpi="0" copies="1"/>
+  <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1"/>
+</x:worksheet>
 </file>
</xml_diff>